<commit_message>
Support multi-feed standard template
</commit_message>
<xml_diff>
--- a/outputs/Standard_Composition_Table.xlsx
+++ b/outputs/Standard_Composition_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wldbs\Desktop\한양인더스트리_정지윤\회사업무\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA9DDB0-F3B3-4545-9FF5-FA29A4C340F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA231FB-3A96-446A-9527-0552B5D83849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14317" yWindow="0" windowWidth="14565" windowHeight="15563" xr2:uid="{1D5846B5-5EC9-4977-A41D-F2775EF472E3}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{1D5846B5-5EC9-4977-A41D-F2775EF472E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Methane</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -49,63 +49,77 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Chemical Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Chemical Fomula</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Molecular Weight</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Water</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>H2O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total Flowrate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>참고 사항</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Total Flowrate kg/hr or Nm3/hr 1가지 입력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. Chemical Name or Chemical Fomula 중 1가지 입력. 단, Chemical Name이 복잡한 경우 Fomula를 기재해야 반응식 및 분자량 자동 계산 가능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. Molecular Weight는 필수 입력칸 아님</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4. mol% or wt% or kg/hr or Nm3/hr 중 1가지 입력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feed 1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Feed 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Oxygen</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nitrogen</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nm3/hr</t>
+  </si>
+  <si>
+    <t>Stream No.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>mol%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>wt%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>kg/hr</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Nm3/hr</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Chemical Name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Chemical Fomula</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Molecular Weight</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Water</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>H2O</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Total Flowrate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>참고 사항</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. Total Flowrate kg/hr or Nm3/hr 1가지 입력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2. Chemical Name or Chemical Fomula 중 1가지 입력. 단, Chemical Name이 복잡한 경우 Fomula를 기재해야 반응식 및 분자량 자동 계산 가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3. Molecular Weight는 필수 입력칸 아님</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4. mol% or wt% or kg/hr or Nm3/hr 중 1가지 입력</t>
+  </si>
+  <si>
+    <t>Feed 3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -169,7 +183,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -177,22 +191,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -201,6 +264,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,121 +626,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D23EB97A-93C9-4AB3-AB6E-2ED95E183ED3}">
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultColWidth="9.59765625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="16.1328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.46484375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.265625" style="1" customWidth="1"/>
-    <col min="4" max="7" width="9.06640625" style="1"/>
-    <col min="8" max="8" width="12.265625" customWidth="1"/>
+    <col min="4" max="7" width="9.59765625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="3" t="s">
+    <row r="6" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7"/>
+      <c r="C7"/>
+    </row>
+    <row r="8" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="4" t="s">
+      <c r="E8" s="11"/>
+      <c r="F8" s="9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="4" t="s">
+      <c r="G8" s="11"/>
+      <c r="H8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="7">
+        <v>2000</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="7">
+        <v>3000</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="7"/>
+      <c r="I9" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="8"/>
+    </row>
+    <row r="12" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="12">
+        <v>16</v>
+      </c>
+      <c r="D12" s="13">
+        <v>90</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+    </row>
+    <row r="13" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="12">
+        <v>18</v>
+      </c>
+      <c r="D13" s="13">
+        <v>10</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+    </row>
+    <row r="14" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="4" t="s">
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13">
+        <v>21</v>
+      </c>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+    </row>
+    <row r="15" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="12" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="4"/>
-    </row>
-    <row r="7" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2">
-        <v>100</v>
-      </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="2">
-        <v>16</v>
-      </c>
-      <c r="D11" s="2">
-        <v>90</v>
-      </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2">
-        <v>18</v>
-      </c>
-      <c r="D12" s="2">
-        <v>10</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13">
+        <v>79</v>
+      </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E9 G9 I9" xr:uid="{757E397C-008F-424E-B92D-86C281F1C7EB}">
+      <formula1>"kg/hr, Nm3/hr"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11 F11 H11" xr:uid="{3B14DF5E-28B0-4645-8009-D013F8D10394}">
+      <formula1>"mol%, wt%, kg/hr, Nm3/hr"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>